<commit_message>
only participant `mock` special uid
</commit_message>
<xml_diff>
--- a/html/app/vbr_metadata_template.xlsx
+++ b/html/app/vbr_metadata_template.xlsx
@@ -12855,10 +12855,10 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="0" showErrorMessage="0" sqref="C2:C1048576" errorTitle="Not in Controlled Vocabulary" error="The value you entered is not in the controlled vocabulary. Contact the HVPCC if additional CV terms are needed.">
       <formula1>'cv'!$B$2:$B$3</formula1>
     </dataValidation>
-    <dataValidation type="textLength" operator="greaterThan" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="D1" promptTitle="Required [cv]" prompt="Race of the participant.">
+    <dataValidation type="textLength" operator="greaterThan" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="D1" promptTitle="Required [cv, list]" prompt="Race of the participant.">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="0" showErrorMessage="1" sqref="D2:D1048576" errorTitle="Not in Controlled Vocabulary" error="The value you entered is not in the controlled vocabulary. Contact the HVPCC if additional CV terms are needed.">
+    <dataValidation type="list" allowBlank="1" showInputMessage="0" showErrorMessage="0" sqref="D2:D1048576" errorTitle="Not in Controlled Vocabulary" error="The value you entered is not in the controlled vocabulary. Contact the HVPCC if additional CV terms are needed.">
       <formula1>'cv'!$C$2:$C$9</formula1>
     </dataValidation>
     <dataValidation type="textLength" operator="greaterThan" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="E1" promptTitle="Required [cv]" prompt="Ethnicity of the participant.">
@@ -12879,10 +12879,10 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="0" showErrorMessage="1" sqref="G2:G1048576" errorTitle="Not in Controlled Vocabulary" error="The value you entered is not in the controlled vocabulary. Contact the HVPCC if additional CV terms are needed.">
       <formula1>'cv'!$F$2:$F$197</formula1>
     </dataValidation>
-    <dataValidation type="textLength" operator="greaterThan" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="H1" promptTitle="Required [cv]" prompt="Country where participant resided during childhood">
+    <dataValidation type="textLength" operator="greaterThan" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="H1" promptTitle="Required [cv, list]" prompt="Country where participant resided during childhood">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="0" showErrorMessage="1" sqref="H2:H1048576" errorTitle="Not in Controlled Vocabulary" error="The value you entered is not in the controlled vocabulary. Contact the HVPCC if additional CV terms are needed.">
+    <dataValidation type="list" allowBlank="1" showInputMessage="0" showErrorMessage="0" sqref="H2:H1048576" errorTitle="Not in Controlled Vocabulary" error="The value you entered is not in the controlled vocabulary. Contact the HVPCC if additional CV terms are needed.">
       <formula1>'cv'!$G$2:$G$197</formula1>
     </dataValidation>
     <dataValidation type="textLength" operator="greaterThan" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="I1" promptTitle="Optional [number]" prompt="Age of pregnancy (in weeks) when participant was born.">
@@ -13330,7 +13330,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="0" showErrorMessage="1" sqref="N2:N1048576" errorTitle="Not in Controlled Vocabulary" error="The value you entered is not in the controlled vocabulary. Contact the HVPCC if additional CV terms are needed.">
       <formula1>'cv'!$Q$2:$Q$5</formula1>
     </dataValidation>
-    <dataValidation type="textLength" operator="greaterThan" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="O1" promptTitle="Optional [ontology]" prompt="NCBI Taxonomy IDs of animals that participant has exposure to. Only the ID (e.g. &quot;NCBI:txid9615&quot;) is needed; the rest of the text is ignored/discarded.">
+    <dataValidation type="textLength" operator="greaterThan" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="O1" promptTitle="Optional [ontology, list]" prompt="NCBI Taxonomy IDs of animals that participant has exposure to. Only the ID (e.g. &quot;NCBI:txid9615&quot;) is needed; the rest of the text is ignored/discarded.">
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="0" showErrorMessage="0" sqref="O2:O1048576" errorTitle="Not in Controlled Vocabulary" error="The value you entered is not in the controlled vocabulary. Contact the HVPCC if additional CV terms are needed.">
@@ -13717,7 +13717,7 @@
     <dataValidation type="textLength" operator="greaterThan" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="B1" promptTitle="Optional [ontology]" prompt="The NCBI BioSample ID associated with this library/processed sample, if this sample has been registered with NCBI. Otherwise, leave this field blank.">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="textLength" operator="greaterThan" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="C1" promptTitle="Conditional [uid]" prompt="`event_uid` is required unless `parent_sample_uid` is provided or `sample_type` is &quot;composite_*&quot;.&#10;&#10;A previously defined event_uid at which this sample was collected. This value must be the same for any sampling that occurred at the same event. May be lef…">
+    <dataValidation type="textLength" operator="greaterThan" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="C1" promptTitle="Conditional [uid]" prompt="`event_uid` is required unless `parent_sample_uid` is provided, `sample_type` is &quot;composite_*&quot;, or `participant_uid` is &quot;mock&quot;.&#10;&#10;A previously defined event_uid at which this sample was collected. This value must be the same for any sampling that occurred…">
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="textLength" operator="greaterThan" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="D1" promptTitle="Required [cv]" prompt="Lab, group, or facility within a grant-level project where the sample was collected and/or processed. This should be the group responsible for metadata about the sample.">

</xml_diff>

<commit_message>
added "kapila" as a `lab` option
</commit_message>
<xml_diff>
--- a/html/app/vbr_metadata_template.xlsx
+++ b/html/app/vbr_metadata_template.xlsx
@@ -3553,7 +3553,7 @@
       </c>
       <c r="AL14" t="inlineStr">
         <is>
-          <t>lareau</t>
+          <t>kapila</t>
         </is>
       </c>
       <c r="AP14" t="inlineStr">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="AZ14" t="inlineStr">
         <is>
-          <t>lareau</t>
+          <t>kapila</t>
         </is>
       </c>
       <c r="BE14" t="inlineStr">
@@ -3690,7 +3690,7 @@
       </c>
       <c r="AL15" t="inlineStr">
         <is>
-          <t>li</t>
+          <t>lareau</t>
         </is>
       </c>
       <c r="AP15" t="inlineStr">
@@ -3720,7 +3720,7 @@
       </c>
       <c r="AZ15" t="inlineStr">
         <is>
-          <t>li</t>
+          <t>lareau</t>
         </is>
       </c>
       <c r="BE15" t="inlineStr">
@@ -3822,7 +3822,7 @@
       </c>
       <c r="AL16" t="inlineStr">
         <is>
-          <t>mason</t>
+          <t>li</t>
         </is>
       </c>
       <c r="AP16" t="inlineStr">
@@ -3852,7 +3852,7 @@
       </c>
       <c r="AZ16" t="inlineStr">
         <is>
-          <t>mason</t>
+          <t>li</t>
         </is>
       </c>
       <c r="BE16" t="inlineStr">
@@ -3954,7 +3954,7 @@
       </c>
       <c r="AL17" t="inlineStr">
         <is>
-          <t>moustafa</t>
+          <t>mason</t>
         </is>
       </c>
       <c r="AP17" t="inlineStr">
@@ -3979,7 +3979,7 @@
       </c>
       <c r="AZ17" t="inlineStr">
         <is>
-          <t>moustafa</t>
+          <t>mason</t>
         </is>
       </c>
       <c r="BE17" t="inlineStr">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="AL18" t="inlineStr">
         <is>
-          <t>naik</t>
+          <t>moustafa</t>
         </is>
       </c>
       <c r="AP18" t="inlineStr">
@@ -4106,7 +4106,7 @@
       </c>
       <c r="AZ18" t="inlineStr">
         <is>
-          <t>naik</t>
+          <t>moustafa</t>
         </is>
       </c>
       <c r="BE18" t="inlineStr">
@@ -4203,7 +4203,7 @@
       </c>
       <c r="AL19" t="inlineStr">
         <is>
-          <t>sabeti</t>
+          <t>naik</t>
         </is>
       </c>
       <c r="AP19" t="inlineStr">
@@ -4228,7 +4228,7 @@
       </c>
       <c r="AZ19" t="inlineStr">
         <is>
-          <t>sabeti</t>
+          <t>naik</t>
         </is>
       </c>
       <c r="BE19" t="inlineStr">
@@ -4325,7 +4325,7 @@
       </c>
       <c r="AL20" t="inlineStr">
         <is>
-          <t>snyder</t>
+          <t>sabeti</t>
         </is>
       </c>
       <c r="AP20" t="inlineStr">
@@ -4350,7 +4350,7 @@
       </c>
       <c r="AZ20" t="inlineStr">
         <is>
-          <t>snyder</t>
+          <t>sabeti</t>
         </is>
       </c>
       <c r="BE20" t="inlineStr">
@@ -4437,7 +4437,7 @@
       </c>
       <c r="AL21" t="inlineStr">
         <is>
-          <t>tcgb</t>
+          <t>snyder</t>
         </is>
       </c>
       <c r="AP21" t="inlineStr">
@@ -4462,7 +4462,7 @@
       </c>
       <c r="AZ21" t="inlineStr">
         <is>
-          <t>tcgb</t>
+          <t>snyder</t>
         </is>
       </c>
       <c r="BE21" t="inlineStr">
@@ -4549,7 +4549,7 @@
       </c>
       <c r="AL22" t="inlineStr">
         <is>
-          <t>yracheta</t>
+          <t>tcgb</t>
         </is>
       </c>
       <c r="AP22" t="inlineStr">
@@ -4574,7 +4574,7 @@
       </c>
       <c r="AZ22" t="inlineStr">
         <is>
-          <t>yracheta</t>
+          <t>tcgb</t>
         </is>
       </c>
       <c r="BE22" t="inlineStr">
@@ -4661,7 +4661,7 @@
       </c>
       <c r="AL23" t="inlineStr">
         <is>
-          <t>zhou</t>
+          <t>yracheta</t>
         </is>
       </c>
       <c r="AP23" t="inlineStr">
@@ -4686,7 +4686,7 @@
       </c>
       <c r="AZ23" t="inlineStr">
         <is>
-          <t>zhou</t>
+          <t>yracheta</t>
         </is>
       </c>
       <c r="BE23" t="inlineStr">
@@ -4771,6 +4771,11 @@
           <t>PCV20 (20-valent Pneumococcal conjugate) [CVX:216]</t>
         </is>
       </c>
+      <c r="AL24" t="inlineStr">
+        <is>
+          <t>zhou</t>
+        </is>
+      </c>
       <c r="AP24" t="inlineStr">
         <is>
           <t xml:space="preserve">  bronchiole [UBERON:0002186]</t>
@@ -4784,6 +4789,11 @@
       <c r="AS24" t="inlineStr">
         <is>
           <t xml:space="preserve">  Sputum specimen container [SNOMED:702223006]</t>
+        </is>
+      </c>
+      <c r="AZ24" t="inlineStr">
+        <is>
+          <t>zhou</t>
         </is>
       </c>
       <c r="BE24" t="inlineStr">
@@ -13722,7 +13732,7 @@
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="0" showErrorMessage="1" sqref="E2:E1048576" errorTitle="Not in Controlled Vocabulary" error="The value you entered is not in the controlled vocabulary. Contact the HVPCC if additional CV terms are needed.">
-      <formula1>'cv'!$AL$2:$AL$23</formula1>
+      <formula1>'cv'!$AL$2:$AL$24</formula1>
     </dataValidation>
     <dataValidation type="textLength" operator="greaterThan" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="F1" promptTitle="Required [cv]" prompt="Indicates the composition of the sample - describes if the sample comes from one participant or is a mixture of material from more than one participant. This field can also include terms for various in vitro or cell culture systems. Contact the HVPCC if …">
       <formula1>0</formula1>
@@ -13991,7 +14001,7 @@
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="0" showErrorMessage="1" sqref="C2:C1048576" errorTitle="Not in Controlled Vocabulary" error="The value you entered is not in the controlled vocabulary. Contact the HVPCC if additional CV terms are needed.">
-      <formula1>'cv'!$AZ$2:$AZ$23</formula1>
+      <formula1>'cv'!$AZ$2:$AZ$24</formula1>
     </dataValidation>
     <dataValidation type="textLength" operator="greaterThan" allowBlank="0" showInputMessage="1" showErrorMessage="1" sqref="D1" promptTitle="Required [yes/no]" prompt="Is this an aliquot, or subsample, of the original library or processed sample?">
       <formula1>0</formula1>

</xml_diff>